<commit_message>
fix: fixes an issue with empty cells (#134)
Co-authored-by: Peter LaValle <peter.lavalle@nhs.net>
</commit_message>
<xml_diff>
--- a/tests/data/passed/workbook.xlsx
+++ b/tests/data/passed/workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/passed/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter.lavalle\Documents\nuh-helper\tests\data\passed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C05CF8E9-B347-DF44-998A-2E52338ACA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD80501-BE62-4C1B-BBF3-5C24F2F9E2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13560" yWindow="2460" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
+    <workbookView xWindow="-3660" yWindow="-20445" windowWidth="24150" windowHeight="18075" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
   </bookViews>
   <sheets>
     <sheet name="page-desc" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>foo</t>
   </si>
@@ -91,6 +91,12 @@
   </si>
   <si>
     <t>nuh71</t>
+  </si>
+  <si>
+    <t>nuh23</t>
+  </si>
+  <si>
+    <t>mushrooms</t>
   </si>
 </sst>
 </file>
@@ -464,19 +470,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E58ABCA7-652D-9640-A447-D695C3291F2E}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -488,10 +494,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640D4E5C-A101-794A-8A66-BA19A027AC5F}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -502,7 +508,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -513,7 +519,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -524,7 +530,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -535,25 +541,34 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C6" s="1">
         <v>42630</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B7" s="1">
         <v>36501</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updates tests - can't hide dates in passthrough tests (oops)
</commit_message>
<xml_diff>
--- a/tests/data/passed/workbook.xlsx
+++ b/tests/data/passed/workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter.lavalle\Documents\nuh-helper\tests\data\passed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/passed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD80501-BE62-4C1B-BBF3-5C24F2F9E2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50F9CE96-C890-A34F-8169-3FC8A9AE81F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3660" yWindow="-20445" windowWidth="24150" windowHeight="18075" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
+    <workbookView xWindow="0" yWindow="21600" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
   </bookViews>
   <sheets>
     <sheet name="page-desc" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>foo</t>
   </si>
@@ -75,9 +75,6 @@
     <t>unknown</t>
   </si>
   <si>
-    <t>2016-07-18 idk</t>
-  </si>
-  <si>
     <t>mssing</t>
   </si>
   <si>
@@ -97,6 +94,12 @@
   </si>
   <si>
     <t>mushrooms</t>
+  </si>
+  <si>
+    <t>this can't be a date - sorry 2016</t>
+  </si>
+  <si>
+    <t>idk - this can't be a date anymore</t>
   </si>
 </sst>
 </file>
@@ -470,19 +473,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E58ABCA7-652D-9640-A447-D695C3291F2E}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -495,9 +498,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640D4E5C-A101-794A-8A66-BA19A027AC5F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -508,7 +511,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -519,9 +522,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1">
         <v>37243</v>
@@ -530,9 +533,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1">
         <v>34240</v>
@@ -541,35 +544,35 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1">
-        <v>42630</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>14</v>
       </c>
       <c r="B7" s="1">
         <v>36501</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: date detection (#130)
Co-authored-by: Peter LaValle <peter.lavalle@nhs.net>
</commit_message>
<xml_diff>
--- a/tests/data/passed/workbook.xlsx
+++ b/tests/data/passed/workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter.lavalle\Documents\nuh-helper\tests\data\passed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/passed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD80501-BE62-4C1B-BBF3-5C24F2F9E2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50F9CE96-C890-A34F-8169-3FC8A9AE81F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3660" yWindow="-20445" windowWidth="24150" windowHeight="18075" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
+    <workbookView xWindow="0" yWindow="21600" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{A8A2A46B-4054-8349-A485-FE3F73A68EB8}"/>
   </bookViews>
   <sheets>
     <sheet name="page-desc" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>foo</t>
   </si>
@@ -75,9 +75,6 @@
     <t>unknown</t>
   </si>
   <si>
-    <t>2016-07-18 idk</t>
-  </si>
-  <si>
     <t>mssing</t>
   </si>
   <si>
@@ -97,6 +94,12 @@
   </si>
   <si>
     <t>mushrooms</t>
+  </si>
+  <si>
+    <t>this can't be a date - sorry 2016</t>
+  </si>
+  <si>
+    <t>idk - this can't be a date anymore</t>
   </si>
 </sst>
 </file>
@@ -470,19 +473,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E58ABCA7-652D-9640-A447-D695C3291F2E}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -495,9 +498,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{640D4E5C-A101-794A-8A66-BA19A027AC5F}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -508,7 +511,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -519,9 +522,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1">
         <v>37243</v>
@@ -530,9 +533,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1">
         <v>34240</v>
@@ -541,35 +544,35 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1">
-        <v>42630</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>14</v>
       </c>
       <c r="B7" s="1">
         <v>36501</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>